<commit_message>
Merge voice + landmark-compare updates (v3 + v4)
web/index.html absorbs both deltas:
- Voice (from v3): voiceQualityScore + FEMALE_VOICE_HINTS heuristic
  picks higher-quality, female-preferring TTS voices per locale,
  with proper exact/prefix/en-fallback chain.
- Compare landmark (from v4): each Compare slot now shows a 16:9
  landmark image (with graceful fallback panel when missing).

Re-mirrors app/index.html, root index.html, terms/index.html from
their site/ and web/ canonicals — the cleanUrls routing reads
those folder duplicates directly.

Bumps pricing across README / LAUNCH_PLAN / BUSINESS_PLAN /
financial_model.xlsx: $7.99/mo, $29.99/yr, Family $49.99/yr.

cap sync run against android/ so the WebView ships the merged
build.

vercel.json and .gitignore deliberately not changed (vercel.json
per task instructions; .gitignore preserves the local Android
public/ exclusion).
</commit_message>
<xml_diff>
--- a/docs/financial_model.xlsx
+++ b/docs/financial_model.xlsx
@@ -862,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="B2:D29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="52" min="2" max="2"/>
@@ -870,7 +870,6 @@
     <col width="40" customWidth="1" style="52" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="33.85" customHeight="1" s="53">
       <c r="B2" s="54" t="inlineStr">
         <is>
@@ -885,7 +884,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="15" customHeight="1" s="53">
       <c r="B5" s="56" t="inlineStr">
         <is>
@@ -893,7 +891,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="53">
       <c r="B7" s="52" t="inlineStr">
         <is>
@@ -935,7 +932,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="53">
       <c r="B11" s="59" t="inlineStr">
         <is>
@@ -1015,8 +1011,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="53">
       <c r="B20" s="59" t="inlineStr">
         <is>
@@ -1045,7 +1039,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="53">
       <c r="B25" s="59" t="inlineStr">
         <is>
@@ -1108,7 +1101,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="53">
       <c r="A3" s="67" t="inlineStr">
         <is>
@@ -1143,7 +1135,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="53">
       <c r="A6" s="67" t="inlineStr">
         <is>
@@ -1251,7 +1242,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="53">
       <c r="A13" s="67" t="inlineStr">
         <is>
@@ -1379,7 +1369,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="53">
       <c r="A21" s="67" t="inlineStr">
         <is>
@@ -1397,10 +1386,10 @@
         <v>3.99</v>
       </c>
       <c r="C22" s="76" t="n">
-        <v>3.99</v>
+        <v>7.99</v>
       </c>
       <c r="D22" s="76" t="n">
-        <v>4.99</v>
+        <v>9.99</v>
       </c>
       <c r="E22" s="77">
         <f>CHOOSE(MATCH(Cover!$C$9,{"Bear","Base","Bull"},0),B22,C22,D22)</f>
@@ -1417,10 +1406,10 @@
         <v>24.99</v>
       </c>
       <c r="C23" s="76" t="n">
-        <v>24.99</v>
+        <v>29.99</v>
       </c>
       <c r="D23" s="76" t="n">
-        <v>29.99</v>
+        <v>39.99</v>
       </c>
       <c r="E23" s="77">
         <f>CHOOSE(MATCH(Cover!$C$9,{"Bear","Base","Bull"},0),B23,C23,D23)</f>
@@ -1437,10 +1426,10 @@
         <v>39.99</v>
       </c>
       <c r="C24" s="76" t="n">
-        <v>39.99</v>
+        <v>49.99</v>
       </c>
       <c r="D24" s="76" t="n">
-        <v>49.99</v>
+        <v>59.99</v>
       </c>
       <c r="E24" s="77">
         <f>CHOOSE(MATCH(Cover!$C$9,{"Bear","Base","Bull"},0),B24,C24,D24)</f>
@@ -1467,7 +1456,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="15" customHeight="1" s="53">
       <c r="A27" s="67" t="inlineStr">
         <is>
@@ -1555,7 +1543,6 @@
         <v/>
       </c>
     </row>
-    <row r="32"/>
     <row r="33" ht="15" customHeight="1" s="53">
       <c r="A33" s="67" t="inlineStr">
         <is>
@@ -1643,7 +1630,6 @@
         <v/>
       </c>
     </row>
-    <row r="38"/>
     <row r="39" ht="15" customHeight="1" s="53">
       <c r="A39" s="67" t="inlineStr">
         <is>
@@ -1751,7 +1737,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
     <row r="46" ht="15" customHeight="1" s="53">
       <c r="A46" s="67" t="inlineStr">
         <is>
@@ -1877,7 +1862,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="53">
       <c r="A3" s="85" t="inlineStr">
         <is>
@@ -2668,7 +2652,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="53">
       <c r="A9" s="85" t="inlineStr">
         <is>
@@ -2820,7 +2803,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="53">
       <c r="A11" s="89" t="inlineStr">
         <is>
@@ -3122,7 +3104,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="53">
       <c r="A14" s="85" t="inlineStr">
         <is>
@@ -3727,7 +3708,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="53">
       <c r="A19" s="85" t="inlineStr">
         <is>
@@ -3873,7 +3853,6 @@
         <v/>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="53">
       <c r="A21" s="90" t="inlineStr">
         <is>
@@ -4052,7 +4031,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="53">
       <c r="A3" s="85" t="inlineStr">
         <is>
@@ -4844,7 +4822,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="53">
       <c r="A9" s="85" t="inlineStr">
         <is>
@@ -5298,7 +5275,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="53">
       <c r="A13" s="94" t="inlineStr">
         <is>
@@ -5477,7 +5453,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="53">
       <c r="A3" s="85" t="inlineStr">
         <is>
@@ -6269,7 +6244,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="53">
       <c r="A9" s="52" t="inlineStr">
         <is>
@@ -6723,7 +6697,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="53">
       <c r="A13" s="52" t="inlineStr">
         <is>
@@ -7479,7 +7452,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="15" customHeight="1" s="53">
       <c r="A19" s="95" t="inlineStr">
         <is>
@@ -7658,7 +7630,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="53">
       <c r="A3" s="85" t="inlineStr">
         <is>
@@ -8148,7 +8119,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="53">
       <c r="A7" s="85" t="inlineStr">
         <is>
@@ -8300,7 +8270,6 @@
         <v/>
       </c>
     </row>
-    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="53">
       <c r="A9" s="90" t="inlineStr">
         <is>
@@ -8485,7 +8454,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="53">
       <c r="A4" s="98" t="inlineStr">
         <is>
@@ -8589,7 +8557,6 @@
         <v/>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="15" customHeight="1" s="53">
       <c r="A10" s="63" t="inlineStr">
         <is>
@@ -8659,7 +8626,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="53">
       <c r="A14" s="59" t="inlineStr">
         <is>
@@ -8683,7 +8649,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16" ht="15" customHeight="1" s="53">
       <c r="A16" s="98" t="inlineStr">
         <is>
@@ -8746,7 +8711,6 @@
         <v/>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="15" customHeight="1" s="53">
       <c r="A23" s="98" t="inlineStr">
         <is>
@@ -8794,7 +8758,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29" ht="15" customHeight="1" s="53">
       <c r="A29" s="98" t="inlineStr">
         <is>

</xml_diff>